<commit_message>
Buat prototype DSS kecil di Python dengan data dummy 40%
</commit_message>
<xml_diff>
--- a/z_ai_mcdm/data-dummy/Data_Dummy_Self_Assessment_IF.xlsx
+++ b/z_ai_mcdm/data-dummy/Data_Dummy_Self_Assessment_IF.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laravel\IF3D-1-SIKOMPU\z_ai_mcdm\data-dummy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5B4043-7AF6-44C5-8A76-0763479DA469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D41220A-1723-4A1B-BF6E-A9F0A949688A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IF" sheetId="1" r:id="rId1"/>
@@ -23,9 +23,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="81">
   <si>
-    <t>Nama Dosen</t>
-  </si>
-  <si>
     <t>NIDN</t>
   </si>
   <si>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>IF630</t>
+  </si>
+  <si>
+    <t>Nama_Dosen</t>
   </si>
 </sst>
 </file>
@@ -697,138 +697,138 @@
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AK1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="AO1" s="3" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1">
         <v>5</v>
@@ -947,13 +947,13 @@
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
@@ -1072,13 +1072,13 @@
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4" s="1">
         <v>6</v>
@@ -1197,13 +1197,13 @@
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" s="1">
         <v>4</v>
@@ -1322,13 +1322,13 @@
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1">
         <v>4</v>
@@ -1447,13 +1447,13 @@
     </row>
     <row r="7" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -1572,13 +1572,13 @@
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" s="1">
         <v>8</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="1">
         <v>3</v>
@@ -1822,13 +1822,13 @@
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" s="1">
         <v>7</v>
@@ -1947,13 +1947,13 @@
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D11" s="1">
         <v>3</v>
@@ -2083,63 +2083,63 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="1">
         <v>5</v>
@@ -2183,13 +2183,13 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
@@ -2233,13 +2233,13 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4" s="1">
         <v>6</v>
@@ -2283,13 +2283,13 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" s="1">
         <v>4</v>
@@ -2333,13 +2333,13 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1">
         <v>4</v>
@@ -2383,13 +2383,13 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -2433,13 +2433,13 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" s="1">
         <v>8</v>
@@ -2483,13 +2483,13 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D9" s="1">
         <v>3</v>
@@ -2533,13 +2533,13 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" s="1">
         <v>7</v>
@@ -2583,13 +2583,13 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D11" s="1">
         <v>3</v>

</xml_diff>